<commit_message>
Bump plugin to 0.14.0: re-sync review generator (v0.7.0), write_summary tool; tighten review calibrations
Checklist-review skill now calls write_summary for the Summary sheet. Also
adds calibrations (extended version-currency search, lsblk ROTA source,
GenAI feature-conditional N/A, hinted-key search) and fixes the GENAI-003
hint in the default checklist template.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/dataiku-diagnosis-checklist-review/resources/checklist_template.xlsx
+++ b/skills/dataiku-diagnosis-checklist-review/resources/checklist_template.xlsx
@@ -4122,7 +4122,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; llmTraceSettings.traceExplorerDefaultWebApp</t>
+          <t>general-settings.json &gt; generativeAISettings &gt; llmTraceSettings.traceExplorerDefaultWebApp</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -4139,7 +4139,7 @@
       <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>llmTraceSettings.traceExplorerDefaultWebApp present in general-settings.json with non-empty projectKey and webAppId fields.</t>
+          <t>generativeAISettings.llmTraceSettings.traceExplorerDefaultWebApp present in general-settings.json with non-empty projectKey and webAppId fields.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Release 0.23.0: re-sync reader 0.5.0, regenerated checklist template, new calibrations and fixtures
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/dataiku-diagnosis-checklist-review/resources/checklist_template.xlsx
+++ b/skills/dataiku-diagnosis-checklist-review/resources/checklist_template.xlsx
@@ -1395,7 +1395,11 @@
           <t>high</t>
         </is>
       </c>
-      <c r="V9" s="3" t="n"/>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
+        </is>
+      </c>
       <c r="W9" s="3" t="n"/>
       <c r="X9" s="3" t="n"/>
       <c r="Y9" s="3" t="n"/>
@@ -7289,7 +7293,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management &gt; Maximum session duration / Idle timeout</t>
+          <t>general-settings.json &gt; security.sessionsMaxTotalTimeMinutes / security.sessionsMaxIdleTimeMinutes (UI: Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -7299,28 +7303,28 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>configured to a finite, non-default timeout value</t>
+          <t>either value set to a finite number of minutes greater than 0</t>
         </is>
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>The source does not mandate a specific numeric threshold, only that admins may configure these fields; treat as satisfied if either or both values are set to a finite duration rather than left unlimited/unset.</t>
+          <t>In general-settings.json a value of 0 means unlimited (the default). The source does not mandate a specific threshold; treat as satisfied if either or both values are greater than 0.</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Diagnosis or exported settings show a configured, finite 'Maximum session duration' and/or 'Idle timeout' value in session management settings.</t>
+          <t>general-settings.json security.sessionsMaxTotalTimeMinutes and/or security.sessionsMaxIdleTimeMinutes is greater than 0.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Session management settings show these fields unset or set to unlimited/no-expiration.</t>
+          <t>Both keys are 0 (unlimited) or absent.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Session management configuration is often not captured in standard diagnostic exports (it's a UI/DB-stored setting, not a config file key); flag as needs_manual_review, noting the source's own caveat about potential lost work from expiring sessions.</t>
+          <t>Flag needs_manual_review only if general-settings.json or its security block is not in the diagnosis; otherwise decide from the two keys. Note the source's caveat that expiring sessions can lose in-progress work.</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
@@ -7355,7 +7359,7 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>No literal config-file key is given for this UI-only setting, and no specific recommended numeric threshold is provided, so the expected_condition is a best-effort conceptual pointer to the UI path rather than a literal field.</t>
+          <t>The source gives only the UI path and no numeric threshold; the file keys were verified against sample bundles, not the source documents.</t>
         </is>
       </c>
       <c r="W4" s="3" t="n"/>
@@ -7402,7 +7406,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management &gt; Force single session per user</t>
+          <t>general-settings.json &gt; security.forceSingleSessionPerUser (UI: Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management &gt; Force single session per user)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -7412,28 +7416,28 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>This is a UI toggle, not a documented general-settings.json/dip.properties key in the source text.</t>
+          <t>Default is false (multiple concurrent sessions allowed).</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Session management settings show 'Force single session per user' enabled.</t>
+          <t>general-settings.json security.forceSingleSessionPerUser is true.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>The setting is shown as disabled (default), allowing multiple concurrent sessions per user.</t>
+          <t>security.forceSingleSessionPerUser is false (default) or absent, allowing multiple concurrent sessions per user.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>This UI-only toggle is often not captured in diagnostic exports; flag as needs_manual_review, noting the default is disabled (multiple sessions allowed).</t>
+          <t>Flag needs_manual_review only if general-settings.json or its security block is not in the diagnosis; otherwise decide from the key.</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
@@ -7468,7 +7472,7 @@
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>No literal config-file key is given for this UI-only setting.</t>
+          <t>The source gives only the UI path; the file key was verified against sample bundles, not the source documents.</t>
         </is>
       </c>
       <c r="W5" s="3" t="n"/>
@@ -8169,34 +8173,34 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>dip.properties &gt; dku.feature.dataTableLinks.enabled</t>
+          <t>general-settings.json &gt; security.disableDataTableLinks, or dip.properties &gt; dku.feature.dataTableLinks.enabled</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>one_of</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>disableDataTableLinks = true, or dataTableLinks.enabled = false</t>
         </is>
       </c>
       <c r="K12" s="3" t="n"/>
       <c r="L12" s="3" t="n"/>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>dip.properties contains dku.feature.dataTableLinks.enabled=false.</t>
+          <t>general-settings.json security.disableDataTableLinks is true, or dip.properties contains dku.feature.dataTableLinks.enabled=false.</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>The key is absent (default true) or explicitly set to true, meaning links in data tables remain clickable.</t>
+          <t>security.disableDataTableLinks is false and the dip.properties key is absent (default: links clickable) or true.</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>If dip.properties content is not present in the diagnosis, flag as needs_manual_review; the default (links clickable) applies absent this key.</t>
+          <t>Check both general-settings.json and dip.properties before flagging needs_manual_review; the default (links clickable) applies when neither sets it.</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">
@@ -8229,7 +8233,11 @@
           <t>high</t>
         </is>
       </c>
-      <c r="V12" s="3" t="n"/>
+      <c r="V12" s="3" t="inlineStr">
+        <is>
+          <t>That disableDataTableLinks is the general-settings counterpart of dku.feature.dataTableLinks.enabled is inferred from the key names; the source documents only the property.</t>
+        </is>
+      </c>
       <c r="W12" s="3" t="n"/>
       <c r="X12" s="3" t="n"/>
       <c r="Y12" s="3" t="n"/>

</xml_diff>